<commit_message>
Split figure generation into one script per figure; add over-triage CI section
- code/figures.py (1 monolithic script, 12 figures) is replaced by figlib.py
  (shared data loading/plotting helpers) plus one standalone, independently
  runnable script per figure/table, orchestrated by run_all.py.
- analysis.py: add Section 11C (over-triage rate vs. each reference standard,
  overall and utilization-critical, with exact 95% CIs) to the Error
  Direction sheet, plus a Study Design reporting-guideline statement.
- Verified byte-for-byte identical output (all figures + workbook) against
  the pre-refactor baseline before committing.
</commit_message>
<xml_diff>
--- a/results/triage_analysis_results.xlsx
+++ b/results/triage_analysis_results.xlsx
@@ -14358,13 +14358,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -14890,6 +14890,346 @@
           <t>Yes</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="14" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>11C: Over-triage Rate vs. Each Reference Standard</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="14" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Over-triage rate = proportion of all cases (not just disagreements) where the LLM decision range was entirely above the reference level. 95% CI is the exact (Clopper–Pearson) interval on the over-triage proportion.</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="14" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="14" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="14" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>N Over-triage</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Over-triage (%)</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="n"/>
+      <c r="G23" s="17" t="n"/>
+      <c r="H23" s="17" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Natural vs. Nurse Triage</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>(9.8%, 18.6%)</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="n"/>
+      <c r="G24" s="14" t="n"/>
+      <c r="H24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Multiturn vs. Nurse Triage</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>(9.8%, 18.6%)</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="n"/>
+      <c r="G25" s="14" t="n"/>
+      <c r="H25" s="14" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Natural vs. Clinician-Adjudicated</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>(13.5%, 23.3%)</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="n"/>
+      <c r="G26" s="14" t="n"/>
+      <c r="H26" s="14" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Multiturn vs. Clinician-Adjudicated</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>23.5%</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>(18.5%, 29.2%)</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="n"/>
+      <c r="G27" s="14" t="n"/>
+      <c r="H27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="n"/>
+      <c r="B28" s="14" t="n"/>
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="14" t="n"/>
+      <c r="G28" s="14" t="n"/>
+      <c r="H28" s="14" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>Utilization-critical over-triage (≥2 steps above reference), with 95% CI</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="14" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>N Over-triage</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Over-triage (%)</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17" t="n"/>
+      <c r="H30" s="17" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Natural vs. Nurse Triage</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>1.6%</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>(0.4%, 4.0%)</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="14" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Multiturn vs. Nurse Triage</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>3.9%</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>(1.9%, 7.1%)</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="14" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Natural vs. Clinician-Adjudicated</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>5.1%</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>(2.7%, 8.6%)</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="14" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Multiturn vs. Clinician-Adjudicated</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="n">
+        <v>255</v>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>7.5%</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>(4.5%, 11.4%)</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="n"/>
+      <c r="G34" s="14" t="n"/>
+      <c r="H34" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>